<commit_message>
arreglé algunos errores míos
</commit_message>
<xml_diff>
--- a/mejores_hiperparametros_xgboost.xlsx
+++ b/mejores_hiperparametros_xgboost.xlsx
@@ -445,19 +445,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>180</v>
+        <v>96</v>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.04714558324780109</v>
+        <v>0.2318382428711447</v>
       </c>
       <c r="D2" t="n">
-        <v>0.143217730057101</v>
+        <v>0.40177526180696</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9940841222253399</v>
+        <v>0.9939798555626117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>